<commit_message>
Add macro-enabled XLSM with single-open category toggle
</commit_message>
<xml_diff>
--- a/indicator_navigation_demo.xlsx
+++ b/indicator_navigation_demo.xlsx
@@ -1380,7 +1380,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1396,6 +1396,8 @@
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="42" customWidth="1" min="13" max="13"/>
+    <col hidden="1" width="12" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1476,6 +1478,12 @@
           <t>Tip: click a Summary indicator to land on a specific detail row.</t>
         </is>
       </c>
+      <c r="N4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O4" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="5" hidden="1" outlineLevel="1">
       <c r="A5" s="3" t="inlineStr">
@@ -1797,6 +1805,12 @@
           <t>Tip: click a Summary indicator to land on a specific detail row.</t>
         </is>
       </c>
+      <c r="N10" t="n">
+        <v>11</v>
+      </c>
+      <c r="O10" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="11" hidden="1" outlineLevel="1">
       <c r="A11" s="3" t="inlineStr">
@@ -2118,6 +2132,12 @@
           <t>Tip: click a Summary indicator to land on a specific detail row.</t>
         </is>
       </c>
+      <c r="N16" t="n">
+        <v>17</v>
+      </c>
+      <c r="O16" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="17" hidden="1" outlineLevel="1">
       <c r="A17" s="3" t="inlineStr">
@@ -2438,6 +2458,12 @@
         <is>
           <t>Tip: click a Summary indicator to land on a specific detail row.</t>
         </is>
+      </c>
+      <c r="N22" t="n">
+        <v>23</v>
+      </c>
+      <c r="O22" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="23" hidden="1" outlineLevel="1">

</xml_diff>